<commit_message>
Remove answer controls from Q10100 materials
</commit_message>
<xml_diff>
--- a/artifacts/任务规格转化.xlsx
+++ b/artifacts/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="Redaa29a541ae456a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R6d8195982b124e40"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -343,7 +343,7 @@
         <x:v>任务ID</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>playwright_account_freeze_release_audit</x:v>
+        <x:v>playwright_account_freeze_release_review</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="32" customHeight="1">
@@ -471,12 +471,12 @@
         <x:v>完成条件</x:v>
       </x:c>
       <x:c r="B18" s="9" t="str">
-        <x:v>npm run audit返回0，六个目标路径可读，四份报告按业务主键闭合</x:v>
+        <x:v>运行入口生成题面所列配置、用例和报告，四份报告按业务主键关联</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="47" customHeight="1">
       <x:c r="A19" s="9" t="str">
-        <x:v>可验证点</x:v>
+        <x:v>业务核对点</x:v>
       </x:c>
       <x:c r="B19" s="9" t="str">
         <x:v>浏览器项目、时区、页面卡片顺序、裁决徽标、按钮状态、TOTP窗口、焦点次序、冻结请求合同与跨报告追溯</x:v>

</xml_diff>